<commit_message>
Changed fees to specifically growth or high growth
</commit_message>
<xml_diff>
--- a/Sources/Manual calc.xlsx
+++ b/Sources/Manual calc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6d20085048815992/Documenti/GitHub/ranking_aus_super/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6d20085048815992/Documenti/GitHub/ranking_aus_super/sources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="483" documentId="8_{6B50DBFC-E840-4F93-9C07-3F647D2188CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9879295D-B0D4-4291-A5D4-B79CC59C9542}"/>
+  <xr:revisionPtr revIDLastSave="698" documentId="8_{6B50DBFC-E840-4F93-9C07-3F647D2188CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE8D6CEC-211C-4326-A9D7-6958909F9201}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{463C025B-1AEA-4D48-A61E-6EBBD6EBE81E}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" activeTab="1" xr2:uid="{463C025B-1AEA-4D48-A61E-6EBBD6EBE81E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="118">
   <si>
     <t>Balance:</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Notes:</t>
   </si>
   <si>
-    <t>0.05% paid from general reserves.</t>
-  </si>
-  <si>
     <t>Dollar fee (per year absolute)</t>
   </si>
   <si>
@@ -117,12 +114,6 @@
     <t>Essential Super_fs7915.pdf</t>
   </si>
   <si>
-    <t>High Growth index</t>
-  </si>
-  <si>
-    <t>https://aware.com.au/member/what-we-offer/fees-and-costs</t>
-  </si>
-  <si>
     <t>MySuper Lifecycle</t>
   </si>
   <si>
@@ -135,9 +126,6 @@
     <t>CareSuper</t>
   </si>
   <si>
-    <t>https://www.caresuper.com.au/members/why-choose-us/fees-and-costs</t>
-  </si>
-  <si>
     <t>Balanced</t>
   </si>
   <si>
@@ -147,15 +135,9 @@
     <t>Brighter Super</t>
   </si>
   <si>
-    <t>MYSUPER</t>
-  </si>
-  <si>
     <t>OneSuper</t>
   </si>
   <si>
-    <t>https://www.superguide.com.au/super-funds-guide/onesuper</t>
-  </si>
-  <si>
     <t>https://www.smartmonday.com.au/tools-and-resources/forms-and-factsheets#pds-smartmonday-prime</t>
   </si>
   <si>
@@ -237,9 +219,6 @@
     <t>MLC Australia</t>
   </si>
   <si>
-    <t>MLC Balanced</t>
-  </si>
-  <si>
     <t>Prime Super</t>
   </si>
   <si>
@@ -273,9 +252,6 @@
     <t>Equipsuper</t>
   </si>
   <si>
-    <t>MySuper</t>
-  </si>
-  <si>
     <t>Equisuper_myfuture-fees-and-other-costs.pdf</t>
   </si>
   <si>
@@ -331,6 +307,93 @@
   </si>
   <si>
     <t>https://www.hesta.com.au/members/your-superannuation/fees-and-costs</t>
+  </si>
+  <si>
+    <t>High Growth</t>
+  </si>
+  <si>
+    <t>iQ Super – For Life</t>
+  </si>
+  <si>
+    <t>Growth Plus</t>
+  </si>
+  <si>
+    <t>High growth</t>
+  </si>
+  <si>
+    <t>Managed Growth</t>
+  </si>
+  <si>
+    <t>MLC High Growth</t>
+  </si>
+  <si>
+    <t>mkspf-fund-offer-combo-kit.pdf</t>
+  </si>
+  <si>
+    <t>Transaction</t>
+  </si>
+  <si>
+    <t>Investment</t>
+  </si>
+  <si>
+    <t>Admin fees</t>
+  </si>
+  <si>
+    <t>Example 50k NGS</t>
+  </si>
+  <si>
+    <t>NESS-Super-Fees-Costs-Guide.pdf</t>
+  </si>
+  <si>
+    <t>1990s Plus</t>
+  </si>
+  <si>
+    <t>HESTA_Fees-and-costs.pdf</t>
+  </si>
+  <si>
+    <t>More-about-First-Super-OCT-2026.pdf</t>
+  </si>
+  <si>
+    <t>Fees from reserves</t>
+  </si>
+  <si>
+    <t>Only has one option</t>
+  </si>
+  <si>
+    <t>ING_DIRECT_Living_Super_Product_Guide.pdf</t>
+  </si>
+  <si>
+    <t>https://www.ing.com.au/superannuation/living-super.html</t>
+  </si>
+  <si>
+    <t>OneSuper ING</t>
+  </si>
+  <si>
+    <t>White labled so ING High Growth</t>
+  </si>
+  <si>
+    <t>https://www.caresuper.com.au/members/advice-and-resources/forms-and-publications/pds-and-tmds</t>
+  </si>
+  <si>
+    <t>Balanced Growth</t>
+  </si>
+  <si>
+    <t>https://aware.com.au/member/contact-aware-super/forms-and-documents/documents#accordion-c3a8965e74-accordion-item</t>
+  </si>
+  <si>
+    <t>MySuper Lifecycle_Future-Saver-PDS.pdf</t>
+  </si>
+  <si>
+    <t>Lifecycle 1990-94</t>
+  </si>
+  <si>
+    <t>CFS High Growth</t>
+  </si>
+  <si>
+    <t>PreMixed High Growth</t>
+  </si>
+  <si>
+    <t>Outlook</t>
   </si>
 </sst>
 </file>
@@ -341,7 +404,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -385,6 +448,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -408,7 +478,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
@@ -421,6 +491,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -776,7 +850,7 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -789,32 +863,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
         <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -822,243 +896,261 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>112</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>31</v>
+      </c>
+      <c r="B10" t="s">
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>88</v>
+      </c>
+      <c r="C13" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="C21" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B31" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C31" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1068,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12160F08-CD7F-42F2-8486-2D3F0ECC06EA}">
-  <dimension ref="A1:AQ20"/>
+  <dimension ref="A1:AQ23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.08984375" bestFit="1" customWidth="1"/>
@@ -1100,100 +1192,100 @@
       <c r="D2" s="10"/>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="B4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
+      <c r="C4" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
         <v>27</v>
       </c>
-      <c r="G4" t="s">
+      <c r="J4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K4" t="s">
         <v>34</v>
       </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>36</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
         <v>40</v>
       </c>
-      <c r="L4" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>44</v>
       </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
         <v>46</v>
       </c>
-      <c r="P4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>52</v>
-      </c>
       <c r="R4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="S4" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="T4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="U4" t="s">
+        <v>58</v>
+      </c>
+      <c r="V4" t="s">
+        <v>59</v>
+      </c>
+      <c r="W4" t="s">
+        <v>61</v>
+      </c>
+      <c r="X4" t="s">
         <v>64</v>
       </c>
-      <c r="V4" t="s">
+      <c r="Y4" t="s">
         <v>66</v>
       </c>
-      <c r="W4" t="s">
-        <v>68</v>
-      </c>
-      <c r="X4" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA4" t="s">
         <v>73</v>
       </c>
-      <c r="Z4" t="s">
-        <v>76</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>81</v>
-      </c>
       <c r="AB4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="AC4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="AD4" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AE4" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="6">
         <f>52*1.1</f>
@@ -1224,7 +1316,7 @@
         <v>67.599999999999994</v>
       </c>
       <c r="J5" s="6">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K5" s="6">
         <v>67.599999999999994</v>
@@ -1237,6 +1329,7 @@
         <v>52</v>
       </c>
       <c r="N5" s="6">
+        <f>78</f>
         <v>78</v>
       </c>
       <c r="O5" s="6">
@@ -1261,8 +1354,7 @@
         <v>65</v>
       </c>
       <c r="U5" s="6">
-        <f>1.15*52</f>
-        <v>59.8</v>
+        <v>60</v>
       </c>
       <c r="V5" s="6">
         <f>1*52</f>
@@ -1312,7 +1404,7 @@
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2">
         <f t="shared" ref="B6:G6" si="0">B5/$B$2</f>
@@ -1348,7 +1440,7 @@
       </c>
       <c r="J6" s="2">
         <f t="shared" si="1"/>
-        <v>1.3333333333333334E-4</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="K6" s="2">
         <f t="shared" si="1"/>
@@ -1392,7 +1484,7 @@
       </c>
       <c r="U6" s="2">
         <f t="shared" si="2"/>
-        <v>3.9866666666666664E-4</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="V6" s="2">
         <f t="shared" si="2"/>
@@ -1464,7 +1556,7 @@
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="F7" s="7">
-        <v>1.6000000000000001E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="G7" s="7">
         <v>1.4E-3</v>
@@ -1500,7 +1592,8 @@
         <v>1.8E-3</v>
       </c>
       <c r="R7" s="7">
-        <v>1.9E-3</v>
+        <f>0.19%+0.014%</f>
+        <v>2.0400000000000001E-3</v>
       </c>
       <c r="S7" s="7">
         <v>1.2750000000000001E-3</v>
@@ -1517,7 +1610,7 @@
       <c r="W7" s="7">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="X7" s="2">
+      <c r="X7" s="7">
         <v>1E-3</v>
       </c>
       <c r="Y7" s="7">
@@ -1576,7 +1669,7 @@
       </c>
       <c r="F8" s="4">
         <f t="shared" si="4"/>
-        <v>1.9466666666666669E-3</v>
+        <v>1.8466666666666666E-3</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" si="4"/>
@@ -1592,7 +1685,7 @@
       </c>
       <c r="J8" s="4">
         <f t="shared" si="5"/>
-        <v>3.6333333333333335E-3</v>
+        <v>3.9000000000000003E-3</v>
       </c>
       <c r="K8" s="4">
         <f t="shared" si="5"/>
@@ -1624,7 +1717,7 @@
       </c>
       <c r="R8" s="4">
         <f t="shared" si="6"/>
-        <v>2.4199999999999998E-3</v>
+        <v>2.5600000000000002E-3</v>
       </c>
       <c r="S8" s="4">
         <f t="shared" si="6"/>
@@ -1636,7 +1729,7 @@
       </c>
       <c r="U8" s="4">
         <f t="shared" si="6"/>
-        <v>1.5986666666666666E-3</v>
+        <v>1.5999999999999999E-3</v>
       </c>
       <c r="V8" s="4">
         <f t="shared" si="6"/>
@@ -1699,10 +1792,10 @@
         <v>3.8999999999999998E-3</v>
       </c>
       <c r="C10" s="8">
-        <v>5.0000000000000001E-3</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="D10" s="8">
-        <v>6.1000000000000004E-3</v>
+        <v>7.3000000000000001E-3</v>
       </c>
       <c r="E10" s="8">
         <v>6.0000000000000001E-3</v>
@@ -1711,10 +1804,10 @@
         <v>4.4000000000000003E-3</v>
       </c>
       <c r="G10" s="8">
-        <v>4.4999999999999997E-3</v>
+        <v>5.1999999999999998E-3</v>
       </c>
       <c r="H10" s="8">
-        <v>6.4999999999999997E-3</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I10" s="8">
         <v>4.7999999999999996E-3</v>
@@ -1726,13 +1819,14 @@
         <v>4.6800000000000001E-3</v>
       </c>
       <c r="L10" s="8">
-        <v>4.3E-3</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="M10" s="8">
-        <v>4.7999999999999996E-3</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="N10" s="8">
-        <v>8.2000000000000007E-3</v>
+        <f>0.53%+0.29%</f>
+        <v>8.199999999999999E-3</v>
       </c>
       <c r="O10" s="8">
         <v>6.1000000000000004E-3</v>
@@ -1747,34 +1841,36 @@
         <v>3.7000000000000002E-3</v>
       </c>
       <c r="S10" s="8">
-        <v>5.4000000000000003E-3</v>
+        <f>0.48%+0.01%</f>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="T10" s="8">
+        <f>0.87%</f>
         <v>8.6999999999999994E-3</v>
       </c>
       <c r="U10" s="8">
-        <v>8.5000000000000006E-3</v>
+        <v>8.3000000000000001E-3</v>
       </c>
       <c r="V10" s="8">
-        <v>3.8E-3</v>
+        <v>3.8999999999999998E-3</v>
       </c>
       <c r="W10" s="8">
         <v>7.1000000000000004E-3</v>
       </c>
       <c r="X10" s="8">
-        <v>4.1999999999999997E-3</v>
+        <v>4.7000000000000002E-3</v>
       </c>
       <c r="Y10" s="8">
         <v>3.8999999999999998E-3</v>
       </c>
       <c r="Z10" s="8">
-        <v>5.1999999999999998E-3</v>
+        <v>5.5999999999999999E-3</v>
       </c>
       <c r="AA10" s="8">
         <v>6.1999999999999998E-3</v>
       </c>
       <c r="AB10" s="8">
-        <v>3.8999999999999998E-3</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="AC10" s="8">
         <v>4.1999999999999997E-3</v>
@@ -1783,7 +1879,7 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AE10" s="8">
-        <v>5.4000000000000003E-3</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="AF10" s="8"/>
       <c r="AG10" s="8"/>
@@ -1806,25 +1902,25 @@
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="C11" s="8">
-        <v>8.9999999999999998E-4</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="D11" s="8">
-        <v>3.7000000000000002E-3</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="E11" s="8">
-        <v>0</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="F11" s="8">
         <v>8.0000000000000004E-4</v>
       </c>
       <c r="G11" s="8">
-        <v>5.0000000000000001E-4</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="H11" s="8">
-        <v>3.3E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="I11" s="8">
-        <v>6.9999999999999999E-4</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="J11" s="8">
         <v>0</v>
@@ -1833,13 +1929,13 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="L11" s="8">
-        <v>8.0000000000000004E-4</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="M11" s="8">
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="N11" s="8">
-        <v>8.9999999999999998E-4</v>
+        <v>1E-3</v>
       </c>
       <c r="O11" s="8">
         <v>8.0000000000000004E-4</v>
@@ -1854,19 +1950,19 @@
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="S11" s="8">
-        <v>5.9999999999999995E-4</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="T11" s="8">
-        <v>1.4E-3</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="U11" s="8">
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="V11" s="8">
-        <v>1.1000000000000001E-3</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="W11" s="8">
-        <v>8.9999999999999998E-4</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="X11" s="8">
         <v>6.9999999999999999E-4</v>
@@ -1915,35 +2011,35 @@
       </c>
       <c r="C13" s="5">
         <f t="shared" si="8"/>
-        <v>7.2466666666666669E-3</v>
+        <v>6.4466666666666665E-3</v>
       </c>
       <c r="D13" s="5">
         <f t="shared" si="8"/>
-        <v>1.0600000000000002E-2</v>
+        <v>8.4999999999999989E-3</v>
       </c>
       <c r="E13" s="5">
         <f t="shared" si="8"/>
-        <v>6.8000000000000005E-3</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="F13" s="5">
         <f t="shared" si="8"/>
-        <v>7.1466666666666675E-3</v>
+        <v>7.0466666666666672E-3</v>
       </c>
       <c r="G13" s="5">
         <f t="shared" si="8"/>
-        <v>6.5733333333333338E-3</v>
+        <v>7.3733333333333324E-3</v>
       </c>
       <c r="H13" s="5">
         <f t="shared" ref="H13:AE13" si="9">H8+H10+H11</f>
-        <v>1.1599999999999999E-2</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="I13" s="5">
         <f t="shared" si="9"/>
-        <v>7.4506666666666662E-3</v>
+        <v>7.5506666666666665E-3</v>
       </c>
       <c r="J13" s="5">
         <f t="shared" si="9"/>
-        <v>6.7333333333333334E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="K13" s="5">
         <f t="shared" si="9"/>
@@ -1951,15 +2047,15 @@
       </c>
       <c r="L13" s="5">
         <f t="shared" si="9"/>
-        <v>7.4720000000000003E-3</v>
+        <v>7.3720000000000001E-3</v>
       </c>
       <c r="M13" s="5">
         <f t="shared" si="9"/>
-        <v>7.0466666666666664E-3</v>
+        <v>7.3466666666666671E-3</v>
       </c>
       <c r="N13" s="5">
         <f t="shared" si="9"/>
-        <v>9.6200000000000001E-3</v>
+        <v>9.7199999999999995E-3</v>
       </c>
       <c r="O13" s="5">
         <f t="shared" si="9"/>
@@ -1975,31 +2071,31 @@
       </c>
       <c r="R13" s="5">
         <f t="shared" si="9"/>
-        <v>6.5200000000000006E-3</v>
+        <v>6.6600000000000001E-3</v>
       </c>
       <c r="S13" s="5">
         <f t="shared" si="9"/>
-        <v>7.7603333333333335E-3</v>
+        <v>6.8603333333333329E-3</v>
       </c>
       <c r="T13" s="5">
         <f t="shared" si="9"/>
-        <v>1.2233333333333334E-2</v>
+        <v>1.1233333333333333E-2</v>
       </c>
       <c r="U13" s="5">
         <f t="shared" si="9"/>
-        <v>1.0398666666666667E-2</v>
+        <v>1.0199999999999999E-2</v>
       </c>
       <c r="V13" s="5">
         <f t="shared" si="9"/>
-        <v>7.7466666666666673E-3</v>
+        <v>8.0466666666666672E-3</v>
       </c>
       <c r="W13" s="5">
         <f t="shared" si="9"/>
-        <v>1.0500000000000001E-2</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="X13" s="5">
         <f t="shared" si="9"/>
-        <v>6.4199999999999995E-3</v>
+        <v>6.9199999999999999E-3</v>
       </c>
       <c r="Y13" s="5">
         <f t="shared" si="9"/>
@@ -2007,7 +2103,7 @@
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>8.8466666666666659E-3</v>
+        <v>9.2466666666666669E-3</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
@@ -2015,7 +2111,7 @@
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>5.1399999999999996E-3</v>
+        <v>5.64E-3</v>
       </c>
       <c r="AC13" s="5">
         <f t="shared" si="9"/>
@@ -2027,7 +2123,7 @@
       </c>
       <c r="AE13" s="5">
         <f t="shared" si="9"/>
-        <v>7.8402666666666666E-3</v>
+        <v>7.5402666666666666E-3</v>
       </c>
       <c r="AF13" s="5"/>
       <c r="AG13" s="5"/>
@@ -2043,67 +2139,253 @@
       <c r="AQ13" s="5"/>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" t="s">
+        <v>109</v>
+      </c>
+      <c r="K14" t="s">
+        <v>105</v>
+      </c>
+      <c r="L14" t="s">
+        <v>79</v>
+      </c>
+      <c r="M14" t="s">
+        <v>89</v>
+      </c>
+      <c r="N14" t="s">
+        <v>79</v>
+      </c>
       <c r="P14" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="Q14" t="s">
-        <v>53</v>
+        <v>47</v>
+      </c>
+      <c r="R14" t="s">
+        <v>101</v>
+      </c>
+      <c r="S14" t="s">
+        <v>89</v>
+      </c>
+      <c r="T14" t="s">
+        <v>79</v>
       </c>
       <c r="U14" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="V14" t="s">
+        <v>93</v>
+      </c>
+      <c r="W14" t="s">
+        <v>79</v>
+      </c>
+      <c r="X14" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>83</v>
+      </c>
+      <c r="AE14" t="s">
         <v>87</v>
       </c>
-      <c r="Z14" t="s">
-        <v>77</v>
-      </c>
-      <c r="AC14" t="s">
-        <v>87</v>
-      </c>
-      <c r="AD14" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" t="s">
-        <v>77</v>
-      </c>
-      <c r="E15" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="T16" t="s">
+        <v>99</v>
+      </c>
       <c r="AB16" s="11"/>
       <c r="AD16" s="11"/>
     </row>
-    <row r="17" spans="28:30" x14ac:dyDescent="0.35">
+    <row r="17" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="J17" s="12">
+        <f>J5</f>
+        <v>60</v>
+      </c>
+      <c r="L17" s="12">
+        <f>L5</f>
+        <v>85.8</v>
+      </c>
+      <c r="M17" s="12">
+        <f>M5</f>
+        <v>52</v>
+      </c>
+      <c r="O17" s="12">
+        <f>O5</f>
+        <v>78</v>
+      </c>
+      <c r="T17" s="12">
+        <f>T5</f>
+        <v>65</v>
+      </c>
+      <c r="Z17" s="12"/>
       <c r="AB17" s="10"/>
+      <c r="AC17" s="10"/>
       <c r="AD17" s="10"/>
     </row>
-    <row r="18" spans="28:30" x14ac:dyDescent="0.35">
+    <row r="18" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="G18" t="s">
+        <v>97</v>
+      </c>
+      <c r="J18" s="13">
+        <f>J10</f>
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="L18" s="13">
+        <f>L10</f>
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="M18" s="13">
+        <v>5.1000000000000004E-3</v>
+      </c>
+      <c r="O18" s="13">
+        <v>6.1000000000000004E-3</v>
+      </c>
+      <c r="T18" s="13">
+        <v>8.6999999999999994E-3</v>
+      </c>
       <c r="AB18" s="10"/>
     </row>
-    <row r="19" spans="28:30" x14ac:dyDescent="0.35">
+    <row r="19" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="G19" t="s">
+        <v>104</v>
+      </c>
+      <c r="J19" s="13">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="L19" s="13">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="M19" s="14">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="O19" s="13"/>
+      <c r="T19" s="13"/>
       <c r="AB19" s="10"/>
-    </row>
-    <row r="20" spans="28:30" x14ac:dyDescent="0.35">
+      <c r="AC19" s="10"/>
+    </row>
+    <row r="20" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="G20" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="13">
+        <f>J7</f>
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="L20" s="13">
+        <f>L7</f>
+        <v>1.8E-3</v>
+      </c>
+      <c r="M20" s="13">
+        <f>M7</f>
+        <v>1.5E-3</v>
+      </c>
+      <c r="O20" s="13">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="T20" s="13">
+        <f>T7</f>
+        <v>1.6999999999999999E-3</v>
+      </c>
       <c r="AB20" s="10"/>
+    </row>
+    <row r="21" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="G21" t="s">
+        <v>96</v>
+      </c>
+      <c r="L21" s="13">
+        <f>L11</f>
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="M21" s="13">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="O21" s="13">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="T21" s="13">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="Z21" s="12"/>
+    </row>
+    <row r="22" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="J22" s="12">
+        <f>50000*SUM(J18:J21)+J17</f>
+        <v>400</v>
+      </c>
+      <c r="L22">
+        <f>50000*SUM(L18:L21)+L17</f>
+        <v>435.79999999999995</v>
+      </c>
+      <c r="M22">
+        <f>50000*SUM(M18:M21)+M17</f>
+        <v>417</v>
+      </c>
+      <c r="O22">
+        <f>50000*SUM(O18:O21)+O17</f>
+        <v>548</v>
+      </c>
+      <c r="T22">
+        <f>50000*SUM(T18:T21)+T17</f>
+        <v>604.99999999999989</v>
+      </c>
+    </row>
+    <row r="23" spans="7:30" x14ac:dyDescent="0.35">
+      <c r="J23">
+        <v>399.2</v>
+      </c>
+      <c r="L23">
+        <v>438.87</v>
+      </c>
+      <c r="M23">
+        <v>417</v>
+      </c>
+      <c r="N23">
+        <v>589.28</v>
+      </c>
+      <c r="T23">
+        <v>625</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>